<commit_message>
Products: client previews Stock sheet + drop invalid UPCs from template
Uploading our own template was importing 0 rows. Two issues:
- Client preview read SheetNames[0] (Instructions), so it parsed 26 garbage
  rows and disabled the Import button. Mirror the server's "Stock" preference.
- The example UPCs in the template failed GS1 check-digit validation, and the
  importer rolls back the whole batch on any error. Blank the UPC cells —
  the column is illustrative, not required.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/barmetrics/public/templates/stock-import-template.xlsx
+++ b/barmetrics/public/templates/stock-import-template.xlsx
@@ -558,7 +558,7 @@
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
     <col min="7" max="7" width="13.83203125" customWidth="1"/>
     <col min="8" max="8" width="17.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -616,7 +616,7 @@
         <v>480</v>
       </c>
       <c r="I2" t="str">
-        <v>619947000018</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -645,7 +645,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>080432400123</v>
+        <v/>
       </c>
     </row>
     <row r="4">

</xml_diff>